<commit_message>
BID RC-V: escreve por extenso os termos abreviados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FuMPiQvjswbB9c7eCTcVzg
</commit_message>
<xml_diff>
--- a/BID-preenchido/BID - RCV  2026 - 2027.xlsx
+++ b/BID-preenchido/BID - RCV  2026 - 2027.xlsx
@@ -4135,10 +4135,10 @@
       <c r="K3" s="100"/>
       <c r="L3" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">AXA: R$ 63.360 (12m) ou R$ 54.490/ano (24m)
-Fairfax: R$ 88.704 (12m) ou R$ 76.032/ano (24m)
-Sura: R$ 266.112 (12m)
-DM 250 mil | DC 350 mil | Contenção 30 mil | Franquia isenta</t>
+          <t xml:space="preserve">AXA: R$ 63.360 (12 meses) ou R$ 54.490 por ano (24 meses)
+Fairfax: R$ 88.704 (12 meses) ou R$ 76.032 por ano (24 meses)
+Sura: R$ 266.112 (12 meses)
+Danos Materiais 250 mil | Danos Corporais 350 mil | Contenção 30 mil | Franquia isenta</t>
         </is>
       </c>
       <c r="M3" s="101" t="inlineStr">
@@ -4172,10 +4172,10 @@
       <c r="K4" s="103"/>
       <c r="L4" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Akad: R$ 5,50/viagem (12m) ou R$ 5,00 (24m)
-AIG: R$ 4,00/viagem (12m) ou R$ 3,50 (24m)
-DM 160 mil | DC 280 mil | Morais 28-30 mil
-Mínimo R$ 350/mês</t>
+          <t xml:space="preserve">Akad: R$ 5,50 por viagem (12 meses) ou R$ 5,00 (24 meses)
+AIG: R$ 4,00 por viagem (12 meses) ou R$ 3,50 (24 meses)
+Danos Materiais 160 mil | Danos Corporais 280 mil | Danos Morais 28 a 30 mil
+Prêmio mínimo R$ 350 por mês</t>
         </is>
       </c>
       <c r="M4" s="101" t="inlineStr">
@@ -4235,8 +4235,8 @@
       <c r="K6" s="106"/>
       <c r="L6" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Essor: ajustável R$ 76.032 (R$ 3,00/viagem) ou averbável R$ 4,00/viagem (mín. R$ 300/mês)
-DM 200 mil | DC 350 mil | Contenção 10 mil</t>
+          <t xml:space="preserve">Essor: ajustável R$ 76.032 (R$ 3,00 por viagem) ou averbável R$ 4,00 por viagem (prêmio mínimo R$ 300 por mês)
+Danos Materiais 200 mil | Danos Corporais 350 mil | Contenção 10 mil</t>
         </is>
       </c>
       <c r="M6" s="100" t="inlineStr">

</xml_diff>